<commit_message>
Make demo links Chrome friendly
</commit_message>
<xml_diff>
--- a/outputs/ochota-prospecting/ochota-prospecting-crm.xlsx
+++ b/outputs/ochota-prospecting/ochota-prospecting-crm.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Raa2fc04dff6b4c08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leady_Ochota" sheetId="2" r:id="R4a65cf580bac4add"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drafty_Maili" sheetId="3" r:id="Rc9dd251dc1384c54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Szablony" sheetId="4" r:id="R884d735238e54499"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zrodla_i_API" sheetId="5" r:id="R9891f0422b054ba7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rebc37ebc4bfe4d30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leady_Ochota" sheetId="2" r:id="R2fd39e757ff240a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drafty_Maili" sheetId="3" r:id="R13d51b1c9f814c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Szablony" sheetId="4" r:id="R452248e4205c4096"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zrodla_i_API" sheetId="5" r:id="R35685658c83743ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -584,7 +584,7 @@
         <x:v>Pon-pt 9:30-17:30; sob 9:30-14:30; niedz. zamknięte</x:v>
       </x:c>
       <x:c r="Q2" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-001</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-001</x:v>
       </x:c>
       <x:c r="R2" t="str">
         <x:v>MarketPortal.pl / StrefaWalut.pl</x:v>
@@ -638,7 +638,7 @@
         <x:v>Całodobowo</x:v>
       </x:c>
       <x:c r="Q3" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-002</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-002</x:v>
       </x:c>
       <x:c r="R3" t="str">
         <x:v>Własna strona / Kantor.Live</x:v>
@@ -688,7 +688,7 @@
         <x:v>Pon-pt 9:00-17:00; sob 10:00-14:00; niedz. zamknięte</x:v>
       </x:c>
       <x:c r="Q4" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-003</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-003</x:v>
       </x:c>
       <x:c r="R4" t="str">
         <x:v>KRS Online</x:v>
@@ -736,7 +736,7 @@
       <x:c r="O5"/>
       <x:c r="P5"/>
       <x:c r="Q5" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-004</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-004</x:v>
       </x:c>
       <x:c r="R5" t="str">
         <x:v>Panorama Firm</x:v>
@@ -782,7 +782,7 @@
       <x:c r="O6"/>
       <x:c r="P6"/>
       <x:c r="Q6" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-005</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-005</x:v>
       </x:c>
       <x:c r="R6" t="str">
         <x:v>Kantroom.pl</x:v>
@@ -828,7 +828,7 @@
       <x:c r="O7"/>
       <x:c r="P7"/>
       <x:c r="Q7" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-006</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-006</x:v>
       </x:c>
       <x:c r="R7" t="str">
         <x:v>Kantroom.pl</x:v>
@@ -874,7 +874,7 @@
       <x:c r="O8"/>
       <x:c r="P8"/>
       <x:c r="Q8" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-007</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-007</x:v>
       </x:c>
       <x:c r="R8" t="str">
         <x:v>Kantroom.pl</x:v>
@@ -951,12 +951,12 @@
         <x:v>Krótka wersja demo strony dla Kantor Akcent</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-001</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-001</x:v>
       </x:c>
       <x:c r="E2" t="str">
         <x:v>Dzień dobry,
 przygotowałem krótką, poglądową wersję nowoczesnej strony dla Kantor Akcent:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-001
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-001
 To nie jest szablon “na sucho” - link pokazuje od razu, jak mogłaby wyglądać strona Państwa kantoru z kursami walut, kalkulatorem, mapą dojazdu oraz sekcją usług typu złoto, srebro i numizmatyka. Wstawiłem już podstawowe dane publiczne: nazwę i lokalizację (ul. Grójecka 95, 02-101 Warszawa).
 Jeżeli obecna strona nie spełnia już swojej roli albo chcieliby Państwo mieć prostą stronę, którą da się szybko aktualizować, mogę przygotować docelową wersję pod Państwa kantor.
 Czy mogę podesłać krótką propozycję wdrożenia albo zadzwonić na 10 minut?
@@ -966,7 +966,7 @@
       <x:c r="F2" t="str">
         <x:v>Dzień dobry,
 wracam tylko z linkiem do poglądowej wersji strony dla Kantor Akcent:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-001
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-001
 Jeżeli temat strony internetowej jest aktualny, mogę dopasować treści, kolory i sekcje pod Państwa realną ofertę oraz przygotować prosty panel do aktualizacji kursów.
 Pozdrawiam,
 Oskar</x:v>
@@ -983,12 +983,12 @@
         <x:v>Krótka wersja demo strony dla Kantor Cris</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-002</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-002</x:v>
       </x:c>
       <x:c r="E3" t="str">
         <x:v>Dzień dobry,
 przygotowałem krótką, poglądową wersję nowoczesnej strony dla Kantor Cris:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-002
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-002
 To nie jest szablon “na sucho” - link pokazuje od razu, jak mogłaby wyglądać strona Państwa kantoru z kursami walut, kalkulatorem, mapą dojazdu oraz sekcją usług typu złoto, srebro i numizmatyka. Wstawiłem już podstawowe dane publiczne: nazwę i lokalizację (ul. Grójecka 42, 02-320 Warszawa).
 Jeżeli obecna strona nie spełnia już swojej roli albo chcieliby Państwo mieć prostą stronę, którą da się szybko aktualizować, mogę przygotować docelową wersję pod Państwa kantor.
 Czy mogę podesłać krótką propozycję wdrożenia albo zadzwonić na 10 minut?
@@ -998,7 +998,7 @@
       <x:c r="F3" t="str">
         <x:v>Dzień dobry,
 wracam tylko z linkiem do poglądowej wersji strony dla Kantor Cris:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-002
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-002
 Jeżeli temat strony internetowej jest aktualny, mogę dopasować treści, kolory i sekcje pod Państwa realną ofertę oraz przygotować prosty panel do aktualizacji kursów.
 Pozdrawiam,
 Oskar</x:v>
@@ -1015,12 +1015,12 @@
         <x:v>Krótka wersja demo strony dla Grysiewicz Ewa. Kantor wymiany walut</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-003</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-003</x:v>
       </x:c>
       <x:c r="E4" t="str">
         <x:v>Dzień dobry,
 przygotowałem krótką, poglądową wersję nowoczesnej strony dla Grysiewicz Ewa. Kantor wymiany walut:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-003
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-003
 To nie jest szablon “na sucho” - link pokazuje od razu, jak mogłaby wyglądać strona Państwa kantoru z kursami walut, kalkulatorem, mapą dojazdu oraz sekcją usług typu złoto, srebro i numizmatyka. Wstawiłem już podstawowe dane publiczne: nazwę i lokalizację (ul. Grójecka 19/25, 02-021 Warszawa).
 Jeżeli obecna strona nie spełnia już swojej roli albo chcieliby Państwo mieć prostą stronę, którą da się szybko aktualizować, mogę przygotować docelową wersję pod Państwa kantor.
 Czy mogę podesłać krótką propozycję wdrożenia albo zadzwonić na 10 minut?
@@ -1030,7 +1030,7 @@
       <x:c r="F4" t="str">
         <x:v>Dzień dobry,
 wracam tylko z linkiem do poglądowej wersji strony dla Grysiewicz Ewa. Kantor wymiany walut:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-003
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-003
 Jeżeli temat strony internetowej jest aktualny, mogę dopasować treści, kolory i sekcje pod Państwa realną ofertę oraz przygotować prosty panel do aktualizacji kursów.
 Pozdrawiam,
 Oskar</x:v>
@@ -1047,12 +1047,12 @@
         <x:v>Krótka wersja demo strony dla Kantor Wymiany Walut - Multiserwis</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-004</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-004</x:v>
       </x:c>
       <x:c r="E5" t="str">
         <x:v>Dzień dobry,
 przygotowałem krótką, poglądową wersję nowoczesnej strony dla Kantor Wymiany Walut - Multiserwis:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-004
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-004
 To nie jest szablon “na sucho” - link pokazuje od razu, jak mogłaby wyglądać strona Państwa kantoru z kursami walut, kalkulatorem, mapą dojazdu oraz sekcją usług typu złoto, srebro i numizmatyka. Wstawiłem już podstawowe dane publiczne: nazwę i lokalizację (Aleje Jerozolimskie 148 (CH Reduta), 02-326 Warszawa).
 Jeżeli obecna strona nie spełnia już swojej roli albo chcieliby Państwo mieć prostą stronę, którą da się szybko aktualizować, mogę przygotować docelową wersję pod Państwa kantor.
 Czy mogę podesłać krótką propozycję wdrożenia albo zadzwonić na 10 minut?
@@ -1062,7 +1062,7 @@
       <x:c r="F5" t="str">
         <x:v>Dzień dobry,
 wracam tylko z linkiem do poglądowej wersji strony dla Kantor Wymiany Walut - Multiserwis:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-004
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-004
 Jeżeli temat strony internetowej jest aktualny, mogę dopasować treści, kolory i sekcje pod Państwa realną ofertę oraz przygotować prosty panel do aktualizacji kursów.
 Pozdrawiam,
 Oskar</x:v>
@@ -1079,12 +1079,12 @@
         <x:v>Krótka wersja demo strony dla Kantor Apollo</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-005</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-005</x:v>
       </x:c>
       <x:c r="E6" t="str">
         <x:v>Dzień dobry,
 przygotowałem krótką, poglądową wersję nowoczesnej strony dla Kantor Apollo:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-005
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-005
 To nie jest szablon “na sucho” - link pokazuje od razu, jak mogłaby wyglądać strona Państwa kantoru z kursami walut, kalkulatorem, mapą dojazdu oraz sekcją usług typu złoto, srebro i numizmatyka. Wstawiłem już podstawowe dane publiczne: nazwę i lokalizację (Aleje Jerozolimskie 179, 02-222 Warszawa).
 Jeżeli obecna strona nie spełnia już swojej roli albo chcieliby Państwo mieć prostą stronę, którą da się szybko aktualizować, mogę przygotować docelową wersję pod Państwa kantor.
 Czy mogę podesłać krótką propozycję wdrożenia albo zadzwonić na 10 minut?
@@ -1094,7 +1094,7 @@
       <x:c r="F6" t="str">
         <x:v>Dzień dobry,
 wracam tylko z linkiem do poglądowej wersji strony dla Kantor Apollo:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-005
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-005
 Jeżeli temat strony internetowej jest aktualny, mogę dopasować treści, kolory i sekcje pod Państwa realną ofertę oraz przygotować prosty panel do aktualizacji kursów.
 Pozdrawiam,
 Oskar</x:v>
@@ -1111,12 +1111,12 @@
         <x:v>Krótka wersja demo strony dla Kantor Fabryka Złota</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-006</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-006</x:v>
       </x:c>
       <x:c r="E7" t="str">
         <x:v>Dzień dobry,
 przygotowałem krótką, poglądową wersję nowoczesnej strony dla Kantor Fabryka Złota:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-006
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-006
 To nie jest szablon “na sucho” - link pokazuje od razu, jak mogłaby wyglądać strona Państwa kantoru z kursami walut, kalkulatorem, mapą dojazdu oraz sekcją usług typu złoto, srebro i numizmatyka. Wstawiłem już podstawowe dane publiczne: nazwę i lokalizację (Aleje Jerozolimskie 179 (CH Blue City), 02-222 Warszawa).
 Jeżeli obecna strona nie spełnia już swojej roli albo chcieliby Państwo mieć prostą stronę, którą da się szybko aktualizować, mogę przygotować docelową wersję pod Państwa kantor.
 Czy mogę podesłać krótką propozycję wdrożenia albo zadzwonić na 10 minut?
@@ -1126,7 +1126,7 @@
       <x:c r="F7" t="str">
         <x:v>Dzień dobry,
 wracam tylko z linkiem do poglądowej wersji strony dla Kantor Fabryka Złota:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-006
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-006
 Jeżeli temat strony internetowej jest aktualny, mogę dopasować treści, kolory i sekcje pod Państwa realną ofertę oraz przygotować prosty panel do aktualizacji kursów.
 Pozdrawiam,
 Oskar</x:v>
@@ -1143,12 +1143,12 @@
         <x:v>Krótka wersja demo strony dla Extrakantor</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-007</x:v>
+        <x:v>https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-007</x:v>
       </x:c>
       <x:c r="E8" t="str">
         <x:v>Dzień dobry,
 przygotowałem krótką, poglądową wersję nowoczesnej strony dla Extrakantor:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-007
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-007
 To nie jest szablon “na sucho” - link pokazuje od razu, jak mogłaby wyglądać strona Państwa kantoru z kursami walut, kalkulatorem, mapą dojazdu oraz sekcją usług typu złoto, srebro i numizmatyka. Wstawiłem już podstawowe dane publiczne: nazwę i lokalizację (Aleje Jerozolimskie 144, Warszawa).
 Jeżeli obecna strona nie spełnia już swojej roli albo chcieliby Państwo mieć prostą stronę, którą da się szybko aktualizować, mogę przygotować docelową wersję pod Państwa kantor.
 Czy mogę podesłać krótką propozycję wdrożenia albo zadzwonić na 10 minut?
@@ -1158,7 +1158,7 @@
       <x:c r="F8" t="str">
         <x:v>Dzień dobry,
 wracam tylko z linkiem do poglądowej wersji strony dla Extrakantor:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-007
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-007
 Jeżeli temat strony internetowej jest aktualny, mogę dopasować treści, kolory i sekcje pod Państwa realną ofertę oraz przygotować prosty panel do aktualizacji kursów.
 Pozdrawiam,
 Oskar</x:v>
@@ -1219,7 +1219,7 @@
       <x:c r="C2" t="str">
         <x:v>Dzień dobry,
 przygotowałem krótką, poglądową wersję nowoczesnej strony dla Kantor Akcent:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-001
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-001
 To nie jest szablon “na sucho” - link pokazuje od razu, jak mogłaby wyglądać strona Państwa kantoru z kursami walut, kalkulatorem, mapą dojazdu oraz sekcją usług typu złoto, srebro i numizmatyka. Wstawiłem już podstawowe dane publiczne: nazwę i lokalizację (ul. Grójecka 95, 02-101 Warszawa).
 Jeżeli obecna strona nie spełnia już swojej roli albo chcieliby Państwo mieć prostą stronę, którą da się szybko aktualizować, mogę przygotować docelową wersję pod Państwa kantor.
 Czy mogę podesłać krótką propozycję wdrożenia albo zadzwonić na 10 minut?
@@ -1237,7 +1237,7 @@
       <x:c r="C3" t="str">
         <x:v>Dzień dobry,
 wracam tylko z linkiem do poglądowej wersji strony dla Kantor Akcent:
-https://oskar-urban.github.io/Kantor-Uniwersalny/#demo-och-001
+https://oskar-urban.github.io/Kantor-Uniwersalny/?d=och-001
 Jeżeli temat strony internetowej jest aktualny, mogę dopasować treści, kolory i sekcje pod Państwa realną ofertę oraz przygotować prosty panel do aktualizacji kursów.
 Pozdrawiam,
 Oskar</x:v>

</xml_diff>